<commit_message>
Flip court grid to courts-as-rows; locals can run on multiple days
- Court view and Excel export: courts as rows, weekdays as columns
- Locals sheet column is now "days" ("Tue, Thu", "Tue/Thu", "Tuesday and
  Thursday"); old single "day" column still reads
- Simulated locals run twice a week like the club's real programs
- Tests for multi-day locals and the legacy column

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wNqCSKMct7SLgzaVgB7ok
</commit_message>
<xml_diff>
--- a/data/sample_input.xlsx
+++ b/data/sample_input.xlsx
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>day</t>
+          <t>days</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Tue, Thu</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Wed</t>
+          <t>Mon, Wed</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1-6</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Tue, Thu</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1352,17 +1352,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Mon, Wed</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5:30</t>
+          <t>3:45</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">

</xml_diff>

<commit_message>
Late-practice exception for 14s-and-under teams (late_ok)
- Teams sheet: late_ok = Yes lets a 14s-and-under team practice at 7:20
  (or the 7 PM weekend block), with a cost so it's only used when needed
- Weekly template requirement is now soft, so a team with no valid
  recurring slot can't make the whole schedule infeasible
- Test for the exception

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wNqCSKMct7SLgzaVgB7ok
</commit_message>
<xml_diff>
--- a/data/sample_input.xlsx
+++ b/data/sample_input.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -430,6 +430,7 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,6 +479,11 @@
           <t>weekend_pref</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>late_ok</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -511,6 +517,7 @@
           <t>AM</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -544,6 +551,7 @@
           <t>AM</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -577,6 +585,7 @@
           <t>AM</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -610,6 +619,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -643,6 +653,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -676,6 +687,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -709,6 +721,7 @@
           <t>AM</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -738,6 +751,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -767,6 +781,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -796,6 +811,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Tournaments (local/travel) and court quality ranking
Tournaments
- New Tournaments sheet and app tab: Local (hosted here) blocks its courts
  all day and the coaches of its locals program; Travel keeps the teams
  going (club + age groups, or listed teams) from practicing on tournament
  days, avoids the day before/after (especially a late practice the night
  before), and prioritizes 2 practices the week leading in
- Shown on the court view, calendar, Excel export, and explained in Review

Court quality
- Courts ranked 1 > 7 > 6 > 5 > 3 > 4 > 2: stage 1 spreads teams across
  times instead of piling onto bad courts (Court 2 last resort); stage 2
  gives the better courts to older and 1s teams (level from "Black"/"Green"
  or a level column)

Tests for both; simulated club includes a travel tournament.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wNqCSKMct7SLgzaVgB7ok
</commit_message>
<xml_diff>
--- a/data/sample_input.xlsx
+++ b/data/sample_input.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Locals" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekends" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closures" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tournaments" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -431,6 +432,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,6 +486,11 @@
           <t>late_ok</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>level</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -518,6 +525,7 @@
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -552,6 +560,7 @@
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -586,6 +595,7 @@
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -620,6 +630,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -654,6 +665,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -688,6 +700,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -722,6 +735,7 @@
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -752,6 +766,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -782,6 +797,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -812,6 +828,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1638,4 +1655,118 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>club</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ages</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>teams</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>program</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>courts</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Boys Travel Tournament</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>11/14/2026</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>11/15/2026</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Boys</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>15-18</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>